<commit_message>
feature: Product based built-in Windows/Linux host health inspection (initialized by team, read-only and non deletable, form → job → report → notification), and complete report template styles and list built-in filtering/viewing, atomic detail viewing.
</commit_message>
<xml_diff>
--- a/web/public/workflow-orchestration/templates/health-inspection-example.xlsx
+++ b/web/public/workflow-orchestration/templates/health-inspection-example.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,12 +39,12 @@
       <name val="Microsoft YaHei"/>
       <b val="1"/>
       <color rgb="001F4E79"/>
-      <sz val="16"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
       <color rgb="0064748B"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
@@ -66,12 +66,23 @@
       <name val="Microsoft YaHei"/>
       <b val="1"/>
       <color rgb="001F4E79"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="00334155"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
       <sz val="10"/>
     </font>
     <font>
@@ -94,12 +105,22 @@
     </font>
     <font>
       <name val="Microsoft YaHei"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -109,6 +130,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,7 +153,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -135,47 +161,70 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -541,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -566,7 +615,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>—— 资源与运行状态审计 ——</t>
+          <t>—— 资源、系统健康与运行状态审计 ——</t>
         </is>
       </c>
     </row>
@@ -616,207 +665,308 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>检查时间</t>
+          <t>主机名</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>{{ r.data.collected_at }}</t>
+          <t>{{ r.data.host.hostname }}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>系统版本</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.data.host.os_version }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>架构</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.data.host.architecture }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>开机时长（小时）</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.data.host.uptime_hours }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>逻辑 CPU</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.data.host.cpu_cores }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>物理内存（GB）</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.data.host.memory_total_gb }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>CPU 热点</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.data.host.top_cpu }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>内存热点</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.data.host.top_memory }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>检查时间</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.data.collected_at }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>检查结论</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>{{ r.data.conclusion }}</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>总体概览</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>指标</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>指标总数</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>{{ r.data.metric_count }}</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>本次采集的检查项</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>严重问题 (Critical)</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>{{ r.data.critical_count }}</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>需立即处理</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>告警问题 (Warning)</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>{{ r.data.warning_count }}</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>建议尽快处理</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>正常项 (Normal)</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>{{ r.data.normal_count }}</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>当前处于正常范围</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>目标总数</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>{{ summary.total }}</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>本次执行主机</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>执行成功</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>{{ summary.succeeded }}</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>脚本执行成功的主机</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>执行失败</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>{{ summary.failed }}</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>脚本执行失败的主机</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>P0 — 立即处理严重项 {{ r.data.critical_count }} 个</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>P1 — 尽快处理告警项 {{ r.data.warning_count }} 个</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>P2 — 持续观察正常项 {{ r.data.normal_count }} 个</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
+          <t>执行成功</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>{{ summary.succeeded }}</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>脚本执行成功的主机</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>执行失败</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>{{ summary.failed }}</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>脚本执行失败的主机</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>P0 — 立即处理严重项 {{ r.data.critical_count }} 个（磁盘/内存/CPU 严重、根只读、临时目录不可写）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>P1 — 尽快处理告警项 {{ r.data.warning_count }} 个（阈值告警、时间同步、服务与防火墙、更新账龄）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>P2 — 持续观察正常项 {{ r.data.normal_count }} 个（含进程热点）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
           <t>— 报告结束 —</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>由 WeOpsX 自动生成 | {{ r.data.collected_at }}</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>由 WeOpsX 自动生成</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>{{ r.data.collected_at }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>{% endfor %}</t>
         </is>
@@ -833,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -846,129 +996,136 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>严重问题</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>{% for r in results %}</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>{% for r in results %}</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>主机</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.target.name }}</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>地址</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.target.ip }}</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.target.operating_system }}</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>主机</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.name }}</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>地址</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.ip }}</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>系统</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.operating_system }}</t>
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>对象</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>分类</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>指标</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>当前值</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>单位</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>健康状态</t>
+        </is>
+      </c>
+      <c r="G4" s="21" t="inlineStr">
+        <is>
+          <t>问题详情</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>对象</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>分类</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>指标</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>当前值</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>单位</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>健康状态</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>问题详情</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>{% for m in r.data.critical|default([]) %}</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>{% for m in r.data.critical|default([]) %}</t>
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.object_name }}</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.category }}</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.display_name|default(m.metric_name) }}</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.value }}</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.unit }}</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.health_status }}</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.detail }}</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.object_name }}</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.category }}</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.metric_name }}</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.value }}</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.unit }}</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.health_status }}</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.detail }}</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>{% endfor %}</t>
         </is>
       </c>
     </row>
@@ -979,14 +1136,10 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>{% endfor %}</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -997,7 +1150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1010,129 +1163,136 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>告警问题</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>{% for r in results %}</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>{% for r in results %}</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>主机</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.target.name }}</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>地址</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.target.ip }}</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.target.operating_system }}</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>主机</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.name }}</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>地址</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.ip }}</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>系统</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.operating_system }}</t>
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>对象</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>分类</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>指标</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>当前值</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>单位</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>健康状态</t>
+        </is>
+      </c>
+      <c r="G4" s="24" t="inlineStr">
+        <is>
+          <t>问题详情</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>对象</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>分类</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>指标</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>当前值</t>
-        </is>
-      </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>单位</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>健康状态</t>
-        </is>
-      </c>
-      <c r="G5" s="16" t="inlineStr">
-        <is>
-          <t>问题详情</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>{% for m in r.data.warning|default([]) %}</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>{% for m in r.data.warning|default([]) %}</t>
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.object_name }}</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.category }}</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.display_name|default(m.metric_name) }}</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.value }}</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.unit }}</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.health_status }}</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.detail }}</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.object_name }}</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.category }}</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.metric_name }}</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.value }}</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.unit }}</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.health_status }}</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.detail }}</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>{% endfor %}</t>
         </is>
       </c>
     </row>
@@ -1143,14 +1303,10 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>{% endfor %}</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1161,7 +1317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1174,129 +1330,136 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>正常项</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>{% for r in results %}</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>{% for r in results %}</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>主机</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.target.name }}</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>地址</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.target.ip }}</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>{{ r.target.operating_system }}</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>主机</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.name }}</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>地址</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.ip }}</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>系统</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.operating_system }}</t>
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>对象</t>
+        </is>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>分类</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>指标</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>当前值</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>单位</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>健康状态</t>
+        </is>
+      </c>
+      <c r="G4" s="26" t="inlineStr">
+        <is>
+          <t>问题详情</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>对象</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>分类</t>
-        </is>
-      </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>指标</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>当前值</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>单位</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>健康状态</t>
-        </is>
-      </c>
-      <c r="G5" s="18" t="inlineStr">
-        <is>
-          <t>问题详情</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>{% for m in r.data.normal|default([]) %}</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>{% for m in r.data.normal|default([]) %}</t>
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.object_name }}</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.category }}</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.display_name|default(m.metric_name) }}</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.value }}</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.unit }}</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.health_status }}</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.detail }}</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.object_name }}</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.category }}</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.metric_name }}</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.value }}</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.unit }}</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.health_status }}</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.detail }}</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>{% endfor %}</t>
         </is>
       </c>
     </row>
@@ -1307,14 +1470,10 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>{% endfor %}</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1325,7 +1484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1340,117 +1499,124 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>检查明细</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>主机</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>对象</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>分类</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>指标</t>
+        </is>
+      </c>
+      <c r="G2" s="28" t="inlineStr">
+        <is>
+          <t>当前值</t>
+        </is>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>健康状态</t>
+        </is>
+      </c>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>主机</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>IP</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>系统</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>对象</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>分类</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>指标</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>当前值</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>健康状态</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>说明</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>{% for r in results %}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>{% for r in results %}</t>
+          <t>{% for m in r.data.metrics|default([]) %}</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>{% for m in r.data.metrics|default([]) %}</t>
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>{{ r.target.name }}</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>{{ r.target.ip }}</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>{{ r.target.operating_system }}</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.object_name }}</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.category }}</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.display_name|default(m.metric_name) }}</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.value }} {{ m.unit }}</t>
+        </is>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.health_status }}</t>
+        </is>
+      </c>
+      <c r="I5" s="22" t="inlineStr">
+        <is>
+          <t>{{ m.detail }}</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.name }}</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.ip }}</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>{{ r.target.operating_system }}</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.object_name }}</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.category }}</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.metric_name }}</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.value }} {{ m.unit }}</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.health_status }}</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>{{ m.detail }}</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>{% endfor %}</t>
         </is>
       </c>
     </row>
@@ -1461,14 +1627,10 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>{% endfor %}</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>